<commit_message>
Sprint 4B - objetivo de compactação por áreas
</commit_message>
<xml_diff>
--- a/outputs/horario_gerado.xlsx
+++ b/outputs/horario_gerado.xlsx
@@ -595,20 +595,20 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
+          <t>GEO
+PROF GEO 3</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>EDF
+PROF EDF 1</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
           <t>MAT
 PROF MAT 1</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>GEO
-PROF GEO 3</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>FTP
-PROF ADM 1</t>
         </is>
       </c>
     </row>
@@ -618,8 +618,8 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>EDF
-PROF EDF 1</t>
+          <t>BIO
+PROF BIO 2</t>
         </is>
       </c>
       <c r="C4" s="5" t="n"/>
@@ -631,24 +631,29 @@
       <c r="A5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="6" t="n"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>FTP
+PROF ADM 1</t>
+        </is>
+      </c>
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
+          <t>FIL
+PROF FIL 2</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
           <t>POR
 PROF POR 1</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>FIL
-PROF FIL 2</t>
-        </is>
-      </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>FIS
-PROF FIS 1</t>
+          <t>QUI
+PROF QUI 1</t>
         </is>
       </c>
     </row>
@@ -656,12 +661,7 @@
       <c r="A6" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>MAT
-PROF MAT 1</t>
-        </is>
-      </c>
+      <c r="B6" s="6" t="n"/>
       <c r="C6" s="6" t="n"/>
       <c r="D6" s="6" t="n"/>
       <c r="E6" s="6" t="n"/>
@@ -671,29 +671,34 @@
       <c r="A7" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>FTP
 PROF ADM 1</t>
         </is>
       </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>MAT
+PROF MAT 1</t>
+        </is>
+      </c>
       <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>HIS
+PROF HIS 3</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>ART
 PROF ART 2</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>HIS
-PROF HIS 3</t>
-        </is>
-      </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>QUI
-PROF QUI 1</t>
+          <t>FIS
+PROF FIS 1</t>
         </is>
       </c>
     </row>
@@ -701,23 +706,18 @@
       <c r="A8" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>BIO
-PROF BIO 2</t>
-        </is>
-      </c>
+      <c r="B8" s="6" t="n"/>
       <c r="C8" s="6" t="n"/>
       <c r="D8" s="3" t="inlineStr">
         <is>
+          <t>SOC
+PROF SOC 2</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
           <t>ING
 PROF ING 2</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>SOC
-PROF SOC 2</t>
         </is>
       </c>
       <c r="F8" s="6" t="n"/>
@@ -735,16 +735,16 @@
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="E5:E6"/>
-    <mergeCell ref="B4:B5"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="C3:C6"/>
+    <mergeCell ref="B7:B8"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="F7:F8"/>
     <mergeCell ref="F5:F6"/>
-    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="B5:B6"/>
     <mergeCell ref="D5:D6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -813,8 +813,8 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>POR
-PROF POR 2</t>
+          <t>ART
+PROF ART 1</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -824,20 +824,20 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>EDF
-PROF EDF 3</t>
+          <t>HIS
+PROF HIS 1</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>BIO
+PROF BIO 1</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>MAT
 PROF MAT 3</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>HIS
-PROF HIS 1</t>
         </is>
       </c>
     </row>
@@ -847,42 +847,47 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>QUI
-PROF QUI 3</t>
+          <t>ING
+PROF ING 1</t>
         </is>
       </c>
       <c r="C4" s="5" t="n"/>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>SOC
 PROF SOC 2</t>
         </is>
       </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>FTP
+PROF MMD 1</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="n"/>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="6" t="n"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>EDF
+PROF EDF 3</t>
+        </is>
+      </c>
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>ART
-PROF ART 1</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>FTP
-PROF MMD 1</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
           <t>FIL
 PROF FIL 1</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>FIS
+PROF FIS 1</t>
         </is>
       </c>
     </row>
@@ -890,19 +895,9 @@
       <c r="A6" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>BIO
-PROF BIO 1</t>
-        </is>
-      </c>
+      <c r="B6" s="6" t="n"/>
       <c r="C6" s="6" t="n"/>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>ING
-PROF ING 1</t>
-        </is>
-      </c>
+      <c r="D6" s="6" t="n"/>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="6" t="n"/>
     </row>
@@ -912,27 +907,27 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>FIS
-PROF FIS 1</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
           <t>POR
 PROF POR 2</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>MAT
 PROF MAT 3</t>
         </is>
       </c>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>GEO
 PROF GEO 2</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>QUI
+PROF QUI 3</t>
         </is>
       </c>
     </row>
@@ -943,7 +938,12 @@
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="6" t="n"/>
       <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>POR
+PROF POR 2</t>
+        </is>
+      </c>
       <c r="F8" s="6" t="n"/>
     </row>
     <row r="11">
@@ -958,17 +958,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="E4:E7"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="E3:E4"/>
     <mergeCell ref="C3:C6"/>
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D3:D4"/>
     <mergeCell ref="D7:D8"/>
+    <mergeCell ref="F3:F4"/>
     <mergeCell ref="F7:F8"/>
     <mergeCell ref="F5:F6"/>
-    <mergeCell ref="E5:E8"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="D5:D6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1036,8 +1036,8 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>FTP
-PROF MMD 1</t>
+          <t>GEO
+PROF GEO 2</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -1047,20 +1047,20 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>FIL
-PROF FIL 1</t>
+          <t>MAT
+PROF MAT 3</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>ART
-PROF ART 1</t>
+          <t>MAT
+PROF MAT 3</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>FIS
-PROF FIS 1</t>
+          <t>BIO
+PROF BIO 1</t>
         </is>
       </c>
     </row>
@@ -1068,51 +1068,61 @@
       <c r="A4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="n"/>
+      <c r="B4" s="6" t="n"/>
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="6" t="n"/>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>ING
-PROF ING 1</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>FTP
+PROF MMD 1</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="n"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>HIS
+PROF HIS 1</t>
+        </is>
+      </c>
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>GEO
-PROF GEO 2</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>POR
-PROF POR 2</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
           <t>QUI
 PROF QUI 3</t>
         </is>
       </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>ART
+PROF ART 1</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n"/>
     </row>
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="6" t="n"/>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>SOC
+PROF SOC 2</t>
+        </is>
+      </c>
       <c r="C6" s="6" t="n"/>
       <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>ING
+PROF ING 1</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="n"/>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -1120,34 +1130,29 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>MAT
-PROF MAT 3</t>
+          <t>FIL
+PROF FIL 1</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>POR
+PROF POR 2</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>FIS
+PROF FIS 1</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>EDF
 PROF EDF 3</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>HIS
-PROF HIS 1</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>MAT
-PROF MAT 3</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>BIO
-PROF BIO 1</t>
-        </is>
-      </c>
+      <c r="F7" s="6" t="n"/>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="2" t="n">
@@ -1155,12 +1160,7 @@
       </c>
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="6" t="n"/>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>SOC
-PROF SOC 2</t>
-        </is>
-      </c>
+      <c r="D8" s="6" t="n"/>
       <c r="E8" s="6" t="n"/>
       <c r="F8" s="3" t="inlineStr">
         <is>
@@ -1181,16 +1181,16 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F4:F7"/>
+    <mergeCell ref="B3:B4"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="E3:E4"/>
     <mergeCell ref="C3:C6"/>
-    <mergeCell ref="B3:B6"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="D3:D4"/>
+    <mergeCell ref="D7:D8"/>
     <mergeCell ref="E7:E8"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="F5:F6"/>
     <mergeCell ref="D5:D6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1270,20 +1270,20 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
+          <t>FTP
+PROF MMD 1</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
           <t>QUI
 PROF QUI 3</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>HIS
-PROF HIS 1</t>
-        </is>
-      </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>FTP
-PROF MMD 1</t>
+          <t>FIL
+PROF FIL 1</t>
         </is>
       </c>
     </row>
@@ -1293,14 +1293,9 @@
       </c>
       <c r="B4" s="6" t="n"/>
       <c r="C4" s="5" t="n"/>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>SOC
-PROF SOC 2</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="2" t="n">
@@ -1313,19 +1308,19 @@
         </is>
       </c>
       <c r="C5" s="5" t="n"/>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>FIS
 PROF FIS 1</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>FIL
-PROF FIL 1</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="n"/>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>GEO
+PROF GEO 2</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="2" t="n">
@@ -1349,26 +1344,26 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
+          <t>EDF
+PROF EDF 3</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>MAT
+PROF MAT 3</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
           <t>POR
 PROF POR 3</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>EDF
-PROF EDF 3</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>GEO
-PROF GEO 2</t>
-        </is>
-      </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>MAT
-PROF MAT 3</t>
+          <t>HIS
+PROF HIS 1</t>
         </is>
       </c>
     </row>
@@ -1382,15 +1377,20 @@
 PROF ING 1</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>BIO
 PROF BIO 1</t>
         </is>
       </c>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="n"/>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>SOC
+PROF SOC 2</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1405,16 +1405,16 @@
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F3:F6"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="E3:E4"/>
     <mergeCell ref="C3:C6"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D3:D6"/>
     <mergeCell ref="D7:D8"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="F5:F6"/>
     <mergeCell ref="B5:B6"/>
-    <mergeCell ref="D5:D6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1482,8 +1482,8 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>QUI
-PROF QUI 4</t>
+          <t>FTP
+PROF MMD 2</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -1492,21 +1492,21 @@
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>GEO
+PROF GEO 2</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>FIS
+PROF FIS 1</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>ART
 PROF ART 1</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>GEO
-PROF GEO 2</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>MAT
-PROF MAT 3</t>
         </is>
       </c>
     </row>
@@ -1514,44 +1514,39 @@
       <c r="A4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="6" t="n"/>
+      <c r="B4" s="5" t="n"/>
       <c r="C4" s="5" t="n"/>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>ING
 PROF ING 1</t>
         </is>
       </c>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>FIS
-PROF FIS 1</t>
-        </is>
-      </c>
+      <c r="B5" s="5" t="n"/>
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>EDF
-PROF EDF 4</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
           <t>HIS
 PROF HIS 1</t>
         </is>
       </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>QUI
+PROF QUI 4</t>
+        </is>
+      </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>FTP
-PROF MMD 2</t>
+          <t>POR
+PROF POR 3</t>
         </is>
       </c>
     </row>
@@ -1561,14 +1556,14 @@
       </c>
       <c r="B6" s="6" t="n"/>
       <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>SOC
 PROF SOC 2</t>
         </is>
       </c>
-      <c r="F6" s="5" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -1576,42 +1571,47 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
+          <t>MAT
+PROF MAT 3</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
           <t>POR
 PROF POR 3</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>FIL
+PROF FIL 3</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>MAT
 PROF MAT 3</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>POR
-PROF POR 3</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>FIL
-PROF FIL 3</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="n"/>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>EDF
+PROF EDF 4</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="2" t="n">
         <v>6</v>
       </c>
       <c r="B8" s="6" t="n"/>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>BIO
 PROF BIO 2</t>
         </is>
       </c>
+      <c r="D8" s="6" t="n"/>
       <c r="E8" s="6" t="n"/>
       <c r="F8" s="6" t="n"/>
     </row>
@@ -1627,17 +1627,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="E5:E6"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="E3:E4"/>
-    <mergeCell ref="F5:F8"/>
     <mergeCell ref="C3:C6"/>
+    <mergeCell ref="B3:B6"/>
+    <mergeCell ref="D3:D4"/>
     <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
     <mergeCell ref="E7:E8"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F5:F6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1705,8 +1705,8 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>FIS
-PROF FIS 1</t>
+          <t>QUI
+PROF QUI 4</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -1715,21 +1715,21 @@
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ART
+PROF ART 1</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>FTP
+PROF MMD 2</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>HIS
 PROF HIS 1</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>FTP
-PROF MMD 2</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>MAT
-PROF MAT 4</t>
         </is>
       </c>
     </row>
@@ -1741,12 +1741,17 @@
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="3" t="inlineStr">
         <is>
+          <t>ING
+PROF ING 1</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
           <t>SOC
 PROF SOC 2</t>
         </is>
       </c>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="6" t="n"/>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="2" t="n">
@@ -1754,22 +1759,22 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>QUI
-PROF QUI 4</t>
+          <t>FIS
+PROF FIS 1</t>
         </is>
       </c>
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
+          <t>POR
+PROF POR 3</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
           <t>FIL
 PROF FIL 3</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>POR
-PROF POR 3</t>
         </is>
       </c>
     </row>
@@ -1789,32 +1794,32 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
+          <t>BIO
+PROF BIO 2</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>EDF
+PROF EDF 4</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
           <t>MAT
 PROF MAT 4</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>BIO
-PROF BIO 2</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>MAT
+PROF MAT 4</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>GEO
 PROF GEO 2</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>ART
-PROF ART 1</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>EDF
-PROF EDF 4</t>
         </is>
       </c>
     </row>
@@ -1822,20 +1827,15 @@
       <c r="A8" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>POR
 PROF POR 3</t>
         </is>
       </c>
+      <c r="C8" s="6" t="n"/>
       <c r="D8" s="6" t="n"/>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>ING
-PROF ING 1</t>
-        </is>
-      </c>
+      <c r="E8" s="6" t="n"/>
       <c r="F8" s="6" t="n"/>
     </row>
     <row r="11">
@@ -1853,10 +1853,10 @@
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="C3:C6"/>
-    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
     <mergeCell ref="D7:D8"/>
     <mergeCell ref="E3:E6"/>
-    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="E7:E8"/>
     <mergeCell ref="F7:F8"/>
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="B5:B6"/>
@@ -1928,31 +1928,31 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>HIS
-PROF HIS 1</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>PROJ</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
           <t>POR
 PROF POR 3</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>PROJ</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>QUI
 PROF QUI 4</t>
         </is>
       </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>MAT
+PROF MAT 4</t>
+        </is>
+      </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>ART
-PROF ART 1</t>
+          <t>FIL
+PROF FIL 3</t>
         </is>
       </c>
     </row>
@@ -1960,21 +1960,11 @@
       <c r="A4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>SOC
-PROF SOC 2</t>
-        </is>
-      </c>
+      <c r="B4" s="6" t="n"/>
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="6" t="n"/>
       <c r="E4" s="6" t="n"/>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>ING
-PROF ING 1</t>
-        </is>
-      </c>
+      <c r="F4" s="6" t="n"/>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="2" t="n">
@@ -1982,27 +1972,27 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>FIL
-PROF FIL 3</t>
+          <t>EDF
+PROF EDF 4</t>
         </is>
       </c>
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
+          <t>FIS
+PROF FIS 3</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
           <t>FTP
 PROF MMD 3</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>FIS
-PROF FIS 3</t>
-        </is>
-      </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>EDF
-PROF EDF 4</t>
+          <t>HIS
+PROF HIS 1</t>
         </is>
       </c>
     </row>
@@ -2012,9 +2002,14 @@
       </c>
       <c r="B6" s="6" t="n"/>
       <c r="C6" s="6" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>SOC
+PROF SOC 2</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -2022,27 +2017,27 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
+          <t>MAT
+PROF MAT 4</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>BIO
+PROF BIO 2</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>ART
+PROF ART 1</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
           <t>GEO
 PROF GEO 4</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>MAT
-PROF MAT 4</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>MAT
-PROF MAT 4</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>POR
-PROF POR 3</t>
         </is>
       </c>
     </row>
@@ -2051,15 +2046,20 @@
         <v>6</v>
       </c>
       <c r="B8" s="6" t="n"/>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>POR
+PROF POR 3</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>ING
+PROF ING 1</t>
+        </is>
+      </c>
       <c r="E8" s="6" t="n"/>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>BIO
-PROF BIO 2</t>
-        </is>
-      </c>
+      <c r="F8" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2073,17 +2073,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="B3:B4"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="C3:C6"/>
     <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
     <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="E5:E8"/>
     <mergeCell ref="B5:B6"/>
-    <mergeCell ref="D5:D8"/>
+    <mergeCell ref="D5:D6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2162,20 +2162,20 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>MAT
-PROF MAT 4</t>
+          <t>FIS
+PROF FIS 3</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>POR
-PROF POR 4</t>
+          <t>HIS
+PROF HIS 1</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>GEO
-PROF GEO 4</t>
+          <t>BIO
+PROF BIO 2</t>
         </is>
       </c>
     </row>
@@ -2188,11 +2188,16 @@
       <c r="D4" s="6" t="n"/>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>BIO
-PROF BIO 2</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="n"/>
+          <t>SOC
+PROF SOC 2</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>POR
+PROF POR 4</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="2" t="n">
@@ -2213,14 +2218,14 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
+          <t>GEO
+PROF GEO 4</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
           <t>FTP
 PROF MMD 3</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>FIL
-PROF FIL 3</t>
         </is>
       </c>
     </row>
@@ -2231,8 +2236,8 @@
       <c r="B6" s="6" t="n"/>
       <c r="C6" s="6" t="n"/>
       <c r="D6" s="6" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="5" t="n"/>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -2240,49 +2245,44 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
+          <t>EDF
+PROF EDF 4</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>MAT
+PROF MAT 4</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
           <t>ART
 PROF ART 2</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>EDF
-PROF EDF 4</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>FIS
-PROF FIS 3</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>HIS
-PROF HIS 1</t>
-        </is>
-      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>FIL
+PROF FIL 3</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="n"/>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>ING
 PROF ING 2</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
       <c r="E8" s="6" t="n"/>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>SOC
-PROF SOC 2</t>
-        </is>
-      </c>
+      <c r="F8" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2296,15 +2296,15 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="E5:E6"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="F5:F8"/>
     <mergeCell ref="C3:C6"/>
+    <mergeCell ref="B7:B8"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="D3:D4"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="E5:E8"/>
+    <mergeCell ref="E7:E8"/>
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="D5:D6"/>
   </mergeCells>
@@ -2374,8 +2374,8 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>FTP
-PROF MMD 3</t>
+          <t>FIS
+PROF FIS 3</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -2384,21 +2384,21 @@
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>QUI
-PROF QUI 4</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>MAT
 PROF MAT 4</t>
         </is>
       </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>GEO
+PROF GEO 4</t>
+        </is>
+      </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>FIL
-PROF FIL 3</t>
+          <t>EDF
+PROF EDF 4</t>
         </is>
       </c>
     </row>
@@ -2406,7 +2406,7 @@
       <c r="A4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="n"/>
+      <c r="B4" s="6" t="n"/>
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="6" t="n"/>
       <c r="E4" s="6" t="n"/>
@@ -2416,24 +2416,29 @@
       <c r="A5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="n"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>BIO
+PROF BIO 2</t>
+        </is>
+      </c>
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>FIS
-PROF FIS 3</t>
+          <t>FTP
+PROF MMD 3</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>FIL
+PROF FIL 3</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>POR
 PROF POR 4</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>HIS
-PROF HIS 1</t>
         </is>
       </c>
     </row>
@@ -2441,49 +2446,39 @@
       <c r="A6" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="6" t="n"/>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>QUI
+PROF QUI 4</t>
+        </is>
+      </c>
       <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
+      <c r="D6" s="5" t="n"/>
       <c r="E6" s="6" t="n"/>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>SOC
-PROF SOC 2</t>
-        </is>
-      </c>
+      <c r="F6" s="6" t="n"/>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>EDF
-PROF EDF 4</t>
-        </is>
-      </c>
+      <c r="B7" s="6" t="n"/>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>POR
-PROF POR 4</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
+          <t>ART
+PROF ART 2</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>HIS
+PROF HIS 1</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>MAT
 PROF MAT 4</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>ART
-PROF ART 2</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>GEO
-PROF GEO 4</t>
         </is>
       </c>
     </row>
@@ -2491,18 +2486,23 @@
       <c r="A8" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="6" t="n"/>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>POR
+PROF POR 4</t>
+        </is>
+      </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>BIO
-PROF BIO 2</t>
+          <t>ING
+PROF ING 2</t>
         </is>
       </c>
       <c r="D8" s="6" t="n"/>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>ING
-PROF ING 2</t>
+          <t>SOC
+PROF SOC 2</t>
         </is>
       </c>
       <c r="F8" s="6" t="n"/>
@@ -2520,16 +2520,16 @@
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="E5:E6"/>
+    <mergeCell ref="B3:B4"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="C3:C6"/>
-    <mergeCell ref="B3:B6"/>
+    <mergeCell ref="F3:F4"/>
     <mergeCell ref="D3:D4"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="F3:F4"/>
     <mergeCell ref="F7:F8"/>
-    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="D5:D8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2597,31 +2597,31 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>FTP
-PROF TI 1</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>PROJ</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
           <t>MAT
 PROF MAT 5</t>
         </is>
       </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>PROJ</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>FIS
+PROF FIS 2</t>
+        </is>
+      </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>FIL
-PROF FIL 2</t>
+          <t>MAT
+PROF MAT 5</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>BIO
-PROF BIO 1</t>
+          <t>HIS
+PROF HIS 2</t>
         </is>
       </c>
     </row>
@@ -2629,14 +2629,14 @@
       <c r="A4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="n"/>
+      <c r="B4" s="6" t="n"/>
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="6" t="n"/>
       <c r="E4" s="6" t="n"/>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>FIS
-PROF FIS 2</t>
+          <t>SOC
+PROF SOC 1</t>
         </is>
       </c>
     </row>
@@ -2644,36 +2644,51 @@
       <c r="A5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="n"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>ART
+PROF ART 1</t>
+        </is>
+      </c>
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>POR
-PROF POR 5</t>
+          <t>BIO
+PROF BIO 1</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>GEO
-PROF GEO 1</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="n"/>
+          <t>FTP
+PROF TI 1</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>FIL
+PROF FIL 2</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="6" t="n"/>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>ING
+PROF ING 1</t>
+        </is>
+      </c>
       <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>QUI
 PROF QUI 2</t>
         </is>
       </c>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="6" t="n"/>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -2681,29 +2696,24 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>MAT
-PROF MAT 5</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
           <t>EDF
 PROF EDF 2</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>ART
-PROF ART 1</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>HIS
-PROF HIS 2</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="n"/>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>POR
+PROF POR 5</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>GEO
+PROF GEO 1</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="2" t="n">
@@ -2713,22 +2723,12 @@
       <c r="C8" s="6" t="n"/>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>ING
-PROF ING 1</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>SOC
-PROF SOC 1</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
           <t>POR
 PROF POR 5</t>
         </is>
       </c>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2742,17 +2742,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="E5:E8"/>
+    <mergeCell ref="B3:B4"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="C3:C6"/>
-    <mergeCell ref="B3:B6"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="D3:D4"/>
-    <mergeCell ref="F6:F7"/>
-    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="D6:D7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2820,8 +2820,8 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>BIO
-PROF BIO 1</t>
+          <t>POR
+PROF POR 5</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -2830,21 +2830,21 @@
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>GEO
-PROF GEO 1</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>MAT
 PROF MAT 5</t>
         </is>
       </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>HIS
+PROF HIS 2</t>
+        </is>
+      </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>MAT
-PROF MAT 5</t>
+          <t>POR
+PROF POR 5</t>
         </is>
       </c>
     </row>
@@ -2852,16 +2852,21 @@
       <c r="A4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>POR
-PROF POR 5</t>
-        </is>
-      </c>
+      <c r="B4" s="6" t="n"/>
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>SOC
+PROF SOC 1</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>BIO
+PROF BIO 1</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="2" t="n">
@@ -2869,27 +2874,27 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
+          <t>FIS
+PROF FIS 2</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>FTP
+PROF TI 1</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>FIL
+PROF FIL 2</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
           <t>ART
 PROF ART 1</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>HIS
-PROF HIS 2</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>QUI
-PROF QUI 2</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>FTP
-PROF TI 1</t>
         </is>
       </c>
     </row>
@@ -2897,21 +2902,16 @@
       <c r="A6" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>ING
 PROF ING 1</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>SOC
-PROF SOC 1</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="5" t="n"/>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -2919,29 +2919,29 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
+          <t>QUI
+PROF QUI 2</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>MAT
+PROF MAT 5</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>GEO
+PROF GEO 1</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
           <t>EDF
 PROF EDF 2</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>POR
-PROF POR 5</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>FIL
-PROF FIL 2</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>FIS
-PROF FIS 2</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="n"/>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="2" t="n">
@@ -2966,16 +2966,16 @@
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="E5:E6"/>
+    <mergeCell ref="B3:B4"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="E3:E4"/>
     <mergeCell ref="C3:C6"/>
     <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
     <mergeCell ref="D3:D4"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
     <mergeCell ref="E7:E8"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="F5:F8"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="D5:D8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3043,31 +3043,31 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
+          <t>HIS
+PROF HIS 3</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>PROJ</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
           <t>MAT
 PROF MAT 1</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>PROJ</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>FIL
-PROF FIL 2</t>
-        </is>
-      </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>ART
-PROF ART 2</t>
+          <t>MAT
+PROF MAT 1</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>POR
-PROF POR 1</t>
+          <t>FTP
+PROF ADM 1</t>
         </is>
       </c>
     </row>
@@ -3075,15 +3075,15 @@
       <c r="A4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="6" t="n"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>SOC
+PROF SOC 2</t>
+        </is>
+      </c>
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="6" t="n"/>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>ING
-PROF ING 2</t>
-        </is>
-      </c>
+      <c r="E4" s="6" t="n"/>
       <c r="F4" s="6" t="n"/>
     </row>
     <row r="5" ht="45" customHeight="1">
@@ -3092,27 +3092,27 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
+          <t>FIL
+PROF FIL 2</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>FIS
+PROF FIS 1</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
           <t>FTP
 PROF ADM 1</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>HIS
-PROF HIS 3</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>FIS
-PROF FIS 1</t>
-        </is>
-      </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>EDF
-PROF EDF 1</t>
+          <t>POR
+PROF POR 1</t>
         </is>
       </c>
     </row>
@@ -3122,12 +3122,7 @@
       </c>
       <c r="B6" s="6" t="n"/>
       <c r="C6" s="6" t="n"/>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>SOC
-PROF SOC 2</t>
-        </is>
-      </c>
+      <c r="D6" s="6" t="n"/>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="n"/>
     </row>
@@ -3137,32 +3132,32 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
+          <t>GEO
+PROF GEO 3</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>EDF
+PROF EDF 1</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>QUI
+PROF QUI 1</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
           <t>BIO
 PROF BIO 2</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>MAT
-PROF MAT 1</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>GEO
-PROF GEO 3</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>QUI
-PROF QUI 1</t>
-        </is>
-      </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>FTP
-PROF ADM 1</t>
+          <t>ART
+PROF ART 2</t>
         </is>
       </c>
     </row>
@@ -3170,16 +3165,21 @@
       <c r="A8" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>POR
 PROF POR 1</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="n"/>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>ING
+PROF ING 2</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3194,17 +3194,17 @@
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="E5:E6"/>
-    <mergeCell ref="B3:B4"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="E3:E4"/>
     <mergeCell ref="C3:C6"/>
+    <mergeCell ref="B7:B8"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
     <mergeCell ref="F3:F4"/>
-    <mergeCell ref="F7:F8"/>
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="B5:B6"/>
+    <mergeCell ref="D5:D6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3272,8 +3272,8 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>MAT
-PROF MAT 5</t>
+          <t>EDF
+PROF EDF 2</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -3283,20 +3283,20 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>HIS
-PROF HIS 2</t>
+          <t>QUI
+PROF QUI 2</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>GEO
+PROF GEO 1</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>FTP
 PROF TI 1</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>EDF
-PROF EDF 2</t>
         </is>
       </c>
     </row>
@@ -3306,14 +3306,9 @@
       </c>
       <c r="B4" s="6" t="n"/>
       <c r="C4" s="5" t="n"/>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>SOC
-PROF SOC 1</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="5" t="n"/>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="2" t="n">
@@ -3321,24 +3316,24 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>QUI
-PROF QUI 2</t>
+          <t>POR
+PROF POR 5</t>
         </is>
       </c>
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>FIL
-PROF FIL 2</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>POR
-PROF POR 5</t>
-        </is>
-      </c>
+          <t>FIS
+PROF FIS 2</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>HIS
+PROF HIS 2</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n"/>
     </row>
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="2" t="n">
@@ -3347,13 +3342,13 @@
       <c r="B6" s="6" t="n"/>
       <c r="C6" s="6" t="n"/>
       <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>ART
-PROF ART 1</t>
-        </is>
-      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>SOC
+PROF SOC 1</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="n"/>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -3361,32 +3356,32 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>FIS
-PROF FIS 2</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
           <t>MAT
 PROF MAT 5</t>
         </is>
       </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>ART
+PROF ART 1</t>
+        </is>
+      </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>GEO
-PROF GEO 1</t>
+          <t>MAT
+PROF MAT 5</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>FIL
+PROF FIL 2</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>POR
 PROF POR 5</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>ING
-PROF ING 1</t>
         </is>
       </c>
     </row>
@@ -3395,7 +3390,12 @@
         <v>6</v>
       </c>
       <c r="B8" s="6" t="n"/>
-      <c r="C8" s="6" t="n"/>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>ING
+PROF ING 1</t>
+        </is>
+      </c>
       <c r="D8" s="6" t="n"/>
       <c r="E8" s="6" t="n"/>
       <c r="F8" s="3" t="inlineStr">
@@ -3417,15 +3417,15 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="F3:F6"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="E3:E4"/>
     <mergeCell ref="C3:C6"/>
     <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D3:D4"/>
     <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E3:E6"/>
     <mergeCell ref="E7:E8"/>
-    <mergeCell ref="F3:F4"/>
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="D5:D6"/>
   </mergeCells>
@@ -3506,20 +3506,20 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>FTP
-PROF TI 2</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>QUI
-PROF QUI 2</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
           <t>POR
 PROF POR 6</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>POR
+PROF POR 6</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>MAT
+PROF MAT 6</t>
         </is>
       </c>
     </row>
@@ -3534,7 +3534,12 @@
         </is>
       </c>
       <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>FTP
+PROF TI 2</t>
+        </is>
+      </c>
       <c r="E4" s="6" t="n"/>
       <c r="F4" s="6" t="n"/>
     </row>
@@ -3552,8 +3557,8 @@
       <c r="D5" s="5" t="n"/>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>FIS
-PROF FIS 2</t>
+          <t>QUI
+PROF QUI 2</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -3569,7 +3574,7 @@
       </c>
       <c r="B6" s="6" t="n"/>
       <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
+      <c r="D6" s="5" t="n"/>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="n"/>
     </row>
@@ -3585,26 +3590,21 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
+          <t>MAT
+PROF MAT 6</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>FIS
+PROF FIS 2</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
           <t>ART
 PROF ART 1</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>BIO
-PROF BIO 1</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>MAT
-PROF MAT 6</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>MAT
-PROF MAT 6</t>
         </is>
       </c>
     </row>
@@ -3613,20 +3613,20 @@
         <v>6</v>
       </c>
       <c r="B8" s="6" t="n"/>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>BIO
+PROF BIO 1</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>ING
 PROF ING 1</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>POR
-PROF POR 6</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3641,14 +3641,14 @@
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="E5:E6"/>
+    <mergeCell ref="D4:D7"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="C3:C6"/>
     <mergeCell ref="B7:B8"/>
-    <mergeCell ref="D3:D6"/>
+    <mergeCell ref="C7:C8"/>
     <mergeCell ref="E7:E8"/>
     <mergeCell ref="F3:F4"/>
-    <mergeCell ref="F7:F8"/>
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="B5:B6"/>
   </mergeCells>
@@ -3718,25 +3718,25 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>ART
-PROF ART 1</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>PROJ</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
           <t>POR
 PROF POR 6</t>
         </is>
       </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>PROJ</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>MAT
+PROF MAT 6</t>
+        </is>
+      </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>BIO
-PROF BIO 1</t>
+          <t>FTP
+PROF TI 2</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -3752,18 +3752,13 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>ING
-PROF ING 1</t>
+          <t>BIO
+PROF BIO 1</t>
         </is>
       </c>
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="6" t="n"/>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>FTP
-PROF TI 2</t>
-        </is>
-      </c>
+      <c r="E4" s="5" t="n"/>
       <c r="F4" s="6" t="n"/>
     </row>
     <row r="5" ht="45" customHeight="1">
@@ -3772,15 +3767,15 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>EDF
-PROF EDF 2</t>
+          <t>QUI
+PROF QUI 2</t>
         </is>
       </c>
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>FIS
-PROF FIS 2</t>
+          <t>ART
+PROF ART 1</t>
         </is>
       </c>
       <c r="E5" s="5" t="n"/>
@@ -3797,8 +3792,13 @@
       </c>
       <c r="B6" s="6" t="n"/>
       <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="5" t="n"/>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>ING
+PROF ING 1</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="n"/>
     </row>
     <row r="7" ht="45" customHeight="1">
@@ -3807,23 +3807,28 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
+          <t>FIS
+PROF FIS 2</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>EDF
+PROF EDF 2</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>POR
+PROF POR 6</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
           <t>MAT
 PROF MAT 6</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>MAT
-PROF MAT 6</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>QUI
-PROF QUI 2</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="n"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
           <t>HIS
@@ -3838,12 +3843,7 @@
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="6" t="n"/>
       <c r="D8" s="6" t="n"/>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>POR
-PROF POR 6</t>
-        </is>
-      </c>
+      <c r="E8" s="6" t="n"/>
       <c r="F8" s="3" t="inlineStr">
         <is>
           <t>SOC
@@ -3863,17 +3863,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="E4:E7"/>
+    <mergeCell ref="F5:F6"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="C3:C6"/>
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E3:E6"/>
+    <mergeCell ref="E7:E8"/>
     <mergeCell ref="F3:F4"/>
-    <mergeCell ref="F5:F6"/>
     <mergeCell ref="B5:B6"/>
-    <mergeCell ref="D5:D6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3952,20 +3952,20 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
+          <t>FIL
+PROF FIL 4</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
           <t>MAT
 PROF MAT 6</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>EDF
-PROF EDF 2</t>
-        </is>
-      </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>FIL
-PROF FIL 4</t>
+          <t>FIS
+PROF FIS 2</t>
         </is>
       </c>
     </row>
@@ -3992,20 +3992,20 @@
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>QUI
-PROF QUI 2</t>
+          <t>GEO
+PROF GEO 3</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>ART
-PROF ART 1</t>
+          <t>EDF
+PROF EDF 2</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>HIS
-PROF HIS 2</t>
+          <t>BIO
+PROF BIO 1</t>
         </is>
       </c>
     </row>
@@ -4016,16 +4016,11 @@
       <c r="B6" s="5" t="n"/>
       <c r="C6" s="6" t="n"/>
       <c r="D6" s="6" t="n"/>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>ING
-PROF ING 1</t>
-        </is>
-      </c>
+      <c r="E6" s="6" t="n"/>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>SOC
-PROF SOC 1</t>
+          <t>QUI
+PROF QUI 2</t>
         </is>
       </c>
     </row>
@@ -4042,22 +4037,17 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>FIS
-PROF FIS 2</t>
+          <t>HIS
+PROF HIS 2</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>POR
-PROF POR 6</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>GEO
-PROF GEO 3</t>
-        </is>
-      </c>
+          <t>ART
+PROF ART 1</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n"/>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="2" t="n">
@@ -4065,14 +4055,24 @@
       </c>
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>SOC
+PROF SOC 1</t>
+        </is>
+      </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>BIO
-PROF BIO 1</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="n"/>
+          <t>ING
+PROF ING 1</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>POR
+PROF POR 6</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4087,15 +4087,15 @@
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="B5:B8"/>
+    <mergeCell ref="E5:E6"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="C3:C6"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="D3:D4"/>
-    <mergeCell ref="D7:D8"/>
     <mergeCell ref="F3:F4"/>
-    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F6:F7"/>
     <mergeCell ref="D5:D6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4164,31 +4164,31 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
+          <t>FTP
+PROF ADM 1</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>PROJ</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>FIS
+PROF FIS 1</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
           <t>FIL
 PROF FIL 2</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>PROJ</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>FIS
-PROF FIS 1</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>POR
-PROF POR 1</t>
-        </is>
-      </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>MAT
-PROF MAT 1</t>
+          <t>EDF
+PROF EDF 1</t>
         </is>
       </c>
     </row>
@@ -4199,12 +4199,7 @@
       <c r="B4" s="6" t="n"/>
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="6" t="n"/>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>MAT
-PROF MAT 1</t>
-        </is>
-      </c>
+      <c r="E4" s="6" t="n"/>
       <c r="F4" s="6" t="n"/>
     </row>
     <row r="5" ht="45" customHeight="1">
@@ -4213,22 +4208,27 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
+          <t>MAT
+PROF MAT 1</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>QUI
+PROF QUI 1</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
           <t>HIS
 PROF HIS 3</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>QUI
-PROF QUI 1</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="n"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>POR
-PROF POR 1</t>
+          <t>ART
+PROF ART 2</t>
         </is>
       </c>
     </row>
@@ -4236,21 +4236,21 @@
       <c r="A6" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>SOC
-PROF SOC 2</t>
-        </is>
-      </c>
+      <c r="B6" s="6" t="n"/>
       <c r="C6" s="6" t="n"/>
       <c r="D6" s="6" t="n"/>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>FTP
-PROF ADM 1</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="n"/>
+          <t>SOC
+PROF SOC 2</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>ING
+PROF ING 2</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -4258,27 +4258,32 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
+          <t>POR
+PROF POR 1</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>FTP
+PROF ADM 1</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>MAT
+PROF MAT 1</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
           <t>GEO
 PROF GEO 3</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>EDF
-PROF EDF 1</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>FTP
-PROF ADM 1</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="n"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>ART
-PROF ART 2</t>
+          <t>BIO
+PROF BIO 2</t>
         </is>
       </c>
     </row>
@@ -4289,16 +4294,11 @@
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="6" t="n"/>
       <c r="D8" s="6" t="n"/>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>BIO
-PROF BIO 2</t>
-        </is>
-      </c>
+      <c r="E8" s="6" t="n"/>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>ING
-PROF ING 2</t>
+          <t>POR
+PROF POR 1</t>
         </is>
       </c>
     </row>
@@ -4316,15 +4316,15 @@
   <mergeCells count="12">
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="E3:E4"/>
     <mergeCell ref="C3:C6"/>
+    <mergeCell ref="B7:B8"/>
     <mergeCell ref="C7:C8"/>
-    <mergeCell ref="B7:B8"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="E7:E8"/>
     <mergeCell ref="F3:F4"/>
-    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="B5:B6"/>
     <mergeCell ref="D5:D6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4404,20 +4404,20 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>POR
-PROF POR 5</t>
+          <t>MAT
+PROF MAT 2</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>FIS
-PROF FIS 2</t>
+          <t>QUI
+PROF QUI 1</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>BIO
-PROF BIO 2</t>
+          <t>ART
+PROF ART 2</t>
         </is>
       </c>
     </row>
@@ -4431,8 +4431,8 @@
       <c r="E4" s="6" t="n"/>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>POR
-PROF POR 5</t>
+          <t>ING
+PROF ING 2</t>
         </is>
       </c>
     </row>
@@ -4455,14 +4455,14 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>QUI
-PROF QUI 1</t>
+          <t>FIS
+PROF FIS 2</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>ART
-PROF ART 2</t>
+          <t>EDF
+PROF EDF 1</t>
         </is>
       </c>
     </row>
@@ -4479,12 +4479,7 @@
       <c r="C6" s="6" t="n"/>
       <c r="D6" s="6" t="n"/>
       <c r="E6" s="6" t="n"/>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>ING
-PROF ING 2</t>
-        </is>
-      </c>
+      <c r="F6" s="6" t="n"/>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -4504,20 +4499,20 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
+          <t>POR
+PROF POR 5</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>POR
+PROF POR 5</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
           <t>MAT
 PROF MAT 2</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>MAT
-PROF MAT 2</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>EDF
-PROF EDF 1</t>
         </is>
       </c>
     </row>
@@ -4527,7 +4522,12 @@
       </c>
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>BIO
+PROF BIO 2</t>
+        </is>
+      </c>
       <c r="E8" s="6" t="n"/>
       <c r="F8" s="6" t="n"/>
     </row>
@@ -4551,9 +4551,9 @@
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="D3:D4"/>
-    <mergeCell ref="D7:D8"/>
     <mergeCell ref="E7:E8"/>
     <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F5:F6"/>
     <mergeCell ref="D5:D6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4622,21 +4622,21 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
+          <t>BIO
+PROF BIO 1</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>PROJ</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
           <t>MAT
 PROF MAT 7</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>PROJ</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>FIS
-PROF FIS 3</t>
-        </is>
-      </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
           <t>FIL
@@ -4645,8 +4645,8 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>MAT
-PROF MAT 7</t>
+          <t>FTP
+PROF IA 1</t>
         </is>
       </c>
     </row>
@@ -4654,11 +4654,16 @@
       <c r="A4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="6" t="n"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>POR
+PROF POR 1</t>
+        </is>
+      </c>
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="6" t="n"/>
       <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
+      <c r="F4" s="5" t="n"/>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="2" t="n">
@@ -4666,29 +4671,24 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>POR
-PROF POR 1</t>
+          <t>QUI
+PROF QUI 3</t>
         </is>
       </c>
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>BIO
-PROF BIO 1</t>
+          <t>ART
+PROF ART 2</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>HIS
-PROF HIS 3</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>FTP
-PROF IA 1</t>
-        </is>
-      </c>
+          <t>GEO
+PROF GEO 1</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n"/>
     </row>
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="2" t="n">
@@ -4698,17 +4698,12 @@
       <c r="C6" s="6" t="n"/>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>QUI
-PROF QUI 3</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>SOC
-PROF SOC 1</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="n"/>
+          <t>ING
+PROF ING 2</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -4716,43 +4711,48 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
+          <t>FIS
+PROF FIS 3</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>MAT
+PROF MAT 7</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>POR
+PROF POR 1</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>HIS
+PROF HIS 3</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
           <t>EDF
 PROF EDF 3</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>ART
-PROF ART 2</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>GEO
-PROF GEO 1</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="n"/>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="2" t="n">
         <v>6</v>
       </c>
       <c r="B8" s="6" t="n"/>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>ING
-PROF ING 2</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>POR
-PROF POR 1</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>SOC
+PROF SOC 1</t>
+        </is>
+      </c>
       <c r="F8" s="6" t="n"/>
     </row>
     <row r="11">
@@ -4767,16 +4767,16 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F3:F6"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="E3:E4"/>
-    <mergeCell ref="F5:F8"/>
     <mergeCell ref="C3:C6"/>
     <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
     <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="F7:F8"/>
     <mergeCell ref="B5:B6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4856,20 +4856,20 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
+          <t>HIS
+PROF HIS 3</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
           <t>FTP
 PROF IA 1</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>FIS
-PROF FIS 3</t>
-        </is>
-      </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>HIS
-PROF HIS 3</t>
+          <t>MAT
+PROF MAT 7</t>
         </is>
       </c>
     </row>
@@ -4879,14 +4879,14 @@
       </c>
       <c r="B4" s="6" t="n"/>
       <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>SOC
 PROF SOC 1</t>
         </is>
       </c>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="6" t="n"/>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="2" t="n">
@@ -4899,17 +4899,17 @@
         </is>
       </c>
       <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>BIO
-PROF BIO 1</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>GEO
 PROF GEO 1</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>QUI
+PROF QUI 3</t>
         </is>
       </c>
     </row>
@@ -4925,12 +4925,7 @@
       </c>
       <c r="C6" s="6" t="n"/>
       <c r="D6" s="6" t="n"/>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>QUI
-PROF QUI 3</t>
-        </is>
-      </c>
+      <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="n"/>
     </row>
     <row r="7" ht="45" customHeight="1">
@@ -4939,27 +4934,32 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
+          <t>MAT
+PROF MAT 7</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
           <t>POR
 PROF POR 4</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>MAT
-PROF MAT 7</t>
-        </is>
-      </c>
       <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>MAT
-PROF MAT 7</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>FIL
 PROF FIL 4</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>POR
+PROF POR 4</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>FIS
+PROF FIS 3</t>
         </is>
       </c>
     </row>
@@ -4968,14 +4968,14 @@
         <v>6</v>
       </c>
       <c r="B8" s="6" t="n"/>
-      <c r="C8" s="6" t="n"/>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>BIO
+PROF BIO 1</t>
+        </is>
+      </c>
       <c r="D8" s="6" t="n"/>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>POR
-PROF POR 4</t>
-        </is>
-      </c>
+      <c r="E8" s="6" t="n"/>
       <c r="F8" s="6" t="n"/>
     </row>
     <row r="11">
@@ -4992,15 +4992,15 @@
   <mergeCells count="11">
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="E3:E4"/>
     <mergeCell ref="C3:C6"/>
-    <mergeCell ref="C7:C8"/>
     <mergeCell ref="B7:B8"/>
-    <mergeCell ref="D3:D6"/>
     <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="E3:E6"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="F3:F4"/>
     <mergeCell ref="F7:F8"/>
     <mergeCell ref="F5:F6"/>
+    <mergeCell ref="D5:D6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5068,25 +5068,25 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>ART
-PROF ART 2</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>PROJ</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
           <t>FIL
 PROF FIL 4</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>PROJ</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>FTP
 PROF IA 1</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>EDF
+PROF EDF 3</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -5100,15 +5100,10 @@
       <c r="A4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>ING
-PROF ING 2</t>
-        </is>
-      </c>
+      <c r="B4" s="6" t="n"/>
       <c r="C4" s="5" t="n"/>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="6" t="n"/>
       <c r="F4" s="6" t="n"/>
     </row>
     <row r="5" ht="45" customHeight="1">
@@ -5117,18 +5112,18 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>EDF
-PROF EDF 3</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
           <t>GEO
 PROF GEO 1</t>
         </is>
       </c>
-      <c r="E5" s="5" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>ART
+PROF ART 2</t>
+        </is>
+      </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
           <t>FIS
@@ -5143,7 +5138,12 @@
       <c r="B6" s="6" t="n"/>
       <c r="C6" s="6" t="n"/>
       <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>ING
+PROF ING 2</t>
+        </is>
+      </c>
       <c r="F6" s="6" t="n"/>
     </row>
     <row r="7" ht="45" customHeight="1">
@@ -5152,20 +5152,20 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
+          <t>HIS
+PROF HIS 3</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>BIO
+PROF BIO 1</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
           <t>MAT
 PROF MAT 7</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>BIO
-PROF BIO 1</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>HIS
-PROF HIS 3</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -5185,19 +5185,19 @@
       <c r="A8" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="6" t="n"/>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>SOC
+PROF SOC 1</t>
+        </is>
+      </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
           <t>POR
 PROF POR 4</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>SOC
-PROF SOC 1</t>
-        </is>
-      </c>
+      <c r="D8" s="6" t="n"/>
       <c r="E8" s="6" t="n"/>
       <c r="F8" s="6" t="n"/>
     </row>
@@ -5213,17 +5213,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B3:B4"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="E3:E4"/>
     <mergeCell ref="C3:C6"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E6"/>
+    <mergeCell ref="D3:D6"/>
+    <mergeCell ref="D7:D8"/>
     <mergeCell ref="E7:E8"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="F7:F8"/>
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="B5:B6"/>
-    <mergeCell ref="D5:D6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5291,8 +5291,8 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>FIL
-PROF FIL 1</t>
+          <t>BIO
+PROF BIO 2</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -5302,20 +5302,20 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>EDF
-PROF EDF 1</t>
+          <t>ART
+PROF ART 2</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>MAT
-PROF MAT 2</t>
+          <t>FTP
+PROF PUB 1</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>POR
-PROF POR 2</t>
+          <t>GEO
+PROF GEO 4</t>
         </is>
       </c>
     </row>
@@ -5323,16 +5323,21 @@
       <c r="A4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="6" t="n"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>POR
+PROF POR 2</t>
+        </is>
+      </c>
       <c r="C4" s="5" t="n"/>
-      <c r="D4" s="6" t="n"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>ING
+PROF ING 2</t>
+        </is>
+      </c>
       <c r="E4" s="6" t="n"/>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>BIO
-PROF BIO 2</t>
-        </is>
-      </c>
+      <c r="F4" s="6" t="n"/>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="2" t="n">
@@ -5340,27 +5345,27 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>GEO
-PROF GEO 4</t>
+          <t>FIS
+PROF FIS 3</t>
         </is>
       </c>
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>MAT
-PROF MAT 2</t>
+          <t>EDF
+PROF EDF 1</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>ART
-PROF ART 2</t>
+          <t>POR
+PROF POR 2</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>QUI
-PROF QUI 1</t>
+          <t>HIS
+PROF HIS 3</t>
         </is>
       </c>
     </row>
@@ -5371,13 +5376,13 @@
       <c r="B6" s="6" t="n"/>
       <c r="C6" s="6" t="n"/>
       <c r="D6" s="6" t="n"/>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>ING
-PROF ING 2</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>SOC
+PROF SOC 1</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -5385,32 +5390,32 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>HIS
-PROF HIS 3</t>
+          <t>QUI
+PROF QUI 1</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>MAT
+PROF MAT 2</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>MAT
+PROF MAT 2</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>FTP
 PROF PUB 1</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>FTP
-PROF PUB 1</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>POR
-PROF POR 2</t>
-        </is>
-      </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>FIS
-PROF FIS 3</t>
+          <t>FIL
+PROF FIL 1</t>
         </is>
       </c>
     </row>
@@ -5418,12 +5423,7 @@
       <c r="A8" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>SOC
-PROF SOC 1</t>
-        </is>
-      </c>
+      <c r="B8" s="6" t="n"/>
       <c r="C8" s="6" t="n"/>
       <c r="D8" s="6" t="n"/>
       <c r="E8" s="6" t="n"/>
@@ -5441,16 +5441,16 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="E5:E6"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="C3:C6"/>
+    <mergeCell ref="B7:B8"/>
     <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D3:D4"/>
     <mergeCell ref="D7:D8"/>
     <mergeCell ref="E7:E8"/>
+    <mergeCell ref="F3:F4"/>
     <mergeCell ref="F7:F8"/>
-    <mergeCell ref="F5:F6"/>
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="D5:D6"/>
   </mergeCells>
@@ -5520,8 +5520,8 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>QUI
-PROF QUI 1</t>
+          <t>FTP
+PROF PUB 1</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -5531,14 +5531,14 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>BIO
-PROF BIO 2</t>
+          <t>FIL
+PROF FIL 1</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>HIS
-PROF HIS 3</t>
+          <t>MAT
+PROF MAT 2</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -5554,18 +5554,8 @@
       </c>
       <c r="B4" s="6" t="n"/>
       <c r="C4" s="5" t="n"/>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>ART
-PROF ART 2</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>SOC
-PROF SOC 1</t>
-        </is>
-      </c>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
       <c r="F4" s="6" t="n"/>
     </row>
     <row r="5" ht="45" customHeight="1">
@@ -5574,27 +5564,27 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>FIS
-PROF FIS 3</t>
+          <t>POR
+PROF POR 2</t>
         </is>
       </c>
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>ING
-PROF ING 2</t>
+          <t>HIS
+PROF HIS 3</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>GEO
-PROF GEO 4</t>
+          <t>QUI
+PROF QUI 1</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>FTP
-PROF PUB 1</t>
+          <t>POR
+PROF POR 2</t>
         </is>
       </c>
     </row>
@@ -5602,12 +5592,17 @@
       <c r="A6" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="6" t="n"/>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>BIO
+PROF BIO 2</t>
+        </is>
+      </c>
       <c r="C6" s="6" t="n"/>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>EDF
-PROF EDF 1</t>
+          <t>SOC
+PROF SOC 1</t>
         </is>
       </c>
       <c r="E6" s="6" t="n"/>
@@ -5619,27 +5614,32 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>POR
-PROF POR 2</t>
+          <t>ART
+PROF ART 2</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>MAT
-PROF MAT 2</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>FIL
-PROF FIL 1</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>FTP
 PROF PUB 1</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>GEO
+PROF GEO 4</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>FIS
+PROF FIS 3</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>EDF
+PROF EDF 1</t>
         </is>
       </c>
     </row>
@@ -5647,14 +5647,14 @@
       <c r="A8" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="6" t="n"/>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>ING
+PROF ING 2</t>
+        </is>
+      </c>
       <c r="C8" s="6" t="n"/>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>POR
-PROF POR 2</t>
-        </is>
-      </c>
+      <c r="D8" s="6" t="n"/>
       <c r="E8" s="6" t="n"/>
       <c r="F8" s="6" t="n"/>
     </row>
@@ -5673,15 +5673,15 @@
     <mergeCell ref="E5:E6"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="E3:E4"/>
     <mergeCell ref="C3:C6"/>
-    <mergeCell ref="B7:B8"/>
     <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="D7:D8"/>
     <mergeCell ref="E7:E8"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="F7:F8"/>
     <mergeCell ref="F5:F6"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="B5:B6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>